<commit_message>
Fixed for in-person experiment with latinsquare
</commit_message>
<xml_diff>
--- a/data_analysis/Participants.xlsx
+++ b/data_analysis/Participants.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfgon\Documents\Postodoc\FittsReaching\data_analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johannavila\Documents\Research\FittsLawR\fittsStudy\data_analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3246E383-1B37-4A85-85E1-23CF96D57946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8AA3D6-135B-46EA-9872-20239E975473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-1150" windowWidth="25820" windowHeight="13900" xr2:uid="{E312E5C9-68AC-4497-BDDB-8740A467E1C4}"/>
+    <workbookView xWindow="31485" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{E312E5C9-68AC-4497-BDDB-8740A467E1C4}"/>
   </bookViews>
   <sheets>
     <sheet name="Participants" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>Order</t>
   </si>
@@ -70,6 +70,9 @@
   </si>
   <si>
     <t>412143b2-afe0-413f-94fa-760dcb890417</t>
+  </si>
+  <si>
+    <t>1356a579-de46-47ba-b38e-3059a66d9154</t>
   </si>
 </sst>
 </file>
@@ -133,8 +136,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{90245000-5E62-4EA6-92CC-73A5CADB4F0B}" name="Table2" displayName="Table2" ref="A1:B10" totalsRowShown="0">
-  <autoFilter ref="A1:B10" xr:uid="{90245000-5E62-4EA6-92CC-73A5CADB4F0B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{90245000-5E62-4EA6-92CC-73A5CADB4F0B}" name="Table2" displayName="Table2" ref="A1:B11" totalsRowShown="0">
+  <autoFilter ref="A1:B11" xr:uid="{90245000-5E62-4EA6-92CC-73A5CADB4F0B}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{71FAC1A9-D0B1-4F4C-9433-2E468D8801B7}" name="Participant id"/>
     <tableColumn id="2" xr3:uid="{DB035266-98F4-40D8-AF2D-38F5FAD9EB9A}" name="Order"/>
@@ -528,7 +531,7 @@
         <v>9</v>
       </c>
       <c r="P6">
-        <v>7128</v>
+        <v>7920</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
@@ -549,7 +552,7 @@
       </c>
       <c r="P7">
         <f>+P6/J10</f>
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
@@ -570,7 +573,7 @@
       </c>
       <c r="P8">
         <f>+P6/PRODUCT(J6)</f>
-        <v>648</v>
+        <v>720</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
@@ -611,6 +614,12 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>1</v>
+      </c>
       <c r="J11">
         <f>+J10*6</f>
         <v>4752</v>
@@ -658,7 +667,7 @@
       </c>
       <c r="B3">
         <f>+COUNTIF(Table2[Order],Total!A3)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>